<commit_message>
feat: add two-way Excel upload and live sync capabilities
</commit_message>
<xml_diff>
--- a/ledgerloom_database.xlsx
+++ b/ledgerloom_database.xlsx
@@ -804,7 +804,7 @@
         <v>cash</v>
       </c>
       <c r="J7" t="str">
-        <v>pending_approval</v>
+        <v>approved</v>
       </c>
       <c r="K7" t="str">
         <v>receipt_ocr</v>
@@ -1081,7 +1081,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1135,9 +1135,35 @@
         <v>success</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AUD-6413</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-10-16T06:55:36.413Z</v>
+      </c>
+      <c r="C3" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D3" t="str">
+        <v>APPROVE_TRANSACTION</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F3" t="str">
+        <v>TX-1006</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Approved transaction TX-1006 amount 15400</v>
+      </c>
+      <c r="H3" t="str">
+        <v>success</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete SME Finance Copilot feature checklist with 30-60-day forecasting, anomaly alert precision, unit economics profitability matrix, and scenario preset switcher
</commit_message>
<xml_diff>
--- a/ledgerloom_database.xlsx
+++ b/ledgerloom_database.xlsx
@@ -804,7 +804,7 @@
         <v>cash</v>
       </c>
       <c r="J7" t="str">
-        <v>approved</v>
+        <v>pending_approval</v>
       </c>
       <c r="K7" t="str">
         <v>receipt_ocr</v>
@@ -1081,7 +1081,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1161,9 +1161,61 @@
         <v>success</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AUD-4006</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-10-16T08:01:34.006Z</v>
+      </c>
+      <c r="C4" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D4" t="str">
+        <v>SWITCH_DEMO_SCENARIO</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F4" t="str">
+        <v>cafe</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Switched demo scenario dataset to BrewCraft Artisan Café (Specialty Coffee)</v>
+      </c>
+      <c r="H4" t="str">
+        <v>success</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>AUD-7891</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-10-16T08:01:47.891Z</v>
+      </c>
+      <c r="C5" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D5" t="str">
+        <v>SWITCH_DEMO_SCENARIO</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F5" t="str">
+        <v>garments</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Switched demo scenario dataset to Loom &amp; Stitch Garments (Factory SME)</v>
+      </c>
+      <c r="H5" t="str">
+        <v>success</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete multi-currency support (BDT, CNY, USD) across all LedgerLoom modules and AI CFO Copilot
</commit_message>
<xml_diff>
--- a/ledgerloom_database.xlsx
+++ b/ledgerloom_database.xlsx
@@ -1081,7 +1081,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1213,9 +1213,113 @@
         <v>success</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AUD-0014</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-10-16T08:47:50.014Z</v>
+      </c>
+      <c r="C6" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D6" t="str">
+        <v>SWITCH_DEMO_SCENARIO</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F6" t="str">
+        <v>cafe</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Switched demo scenario dataset to BrewCraft Artisan Café (Specialty Coffee)</v>
+      </c>
+      <c r="H6" t="str">
+        <v>success</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AUD-3174</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-10-16T08:47:53.174Z</v>
+      </c>
+      <c r="C7" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D7" t="str">
+        <v>SWITCH_DEMO_SCENARIO</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F7" t="str">
+        <v>garments</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Switched demo scenario dataset to Loom &amp; Stitch Garments (Factory SME)</v>
+      </c>
+      <c r="H7" t="str">
+        <v>success</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AUD-1406</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-10-16T08:48:01.406Z</v>
+      </c>
+      <c r="C8" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D8" t="str">
+        <v>SWITCH_DEMO_SCENARIO</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F8" t="str">
+        <v>cafe</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Switched demo scenario dataset to BrewCraft Artisan Café (Specialty Coffee)</v>
+      </c>
+      <c r="H8" t="str">
+        <v>success</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AUD-2509</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-10-16T08:48:02.509Z</v>
+      </c>
+      <c r="C9" t="str">
+        <v>owner</v>
+      </c>
+      <c r="D9" t="str">
+        <v>SWITCH_DEMO_SCENARIO</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Tier-4-Execute</v>
+      </c>
+      <c r="F9" t="str">
+        <v>garments</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Switched demo scenario dataset to Loom &amp; Stitch Garments (Factory SME)</v>
+      </c>
+      <c r="H9" t="str">
+        <v>success</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>